<commit_message>
Posts Facebook e melhora nos códigos
</commit_message>
<xml_diff>
--- a/dados/ig_comentarios.xlsx
+++ b/dados/ig_comentarios.xlsx
@@ -49,211 +49,211 @@
     <t>owner</t>
   </si>
   <si>
+    <t>https://www.instagram.com/napucminas/p/DY5JQwiEeiq/</t>
+  </si>
+  <si>
     <t>https://www.instagram.com/napucminas/p/DY2y0nlyyo1/</t>
   </si>
   <si>
-    <t>https://www.instagram.com/napucminas/p/DY5JQwiEeiq/</t>
-  </si>
-  <si>
-    <t>https://www.instagram.com/p/DY2y0nlyyo1/c/17930061063295835</t>
-  </si>
-  <si>
-    <t>https://www.instagram.com/p/DY2y0nlyyo1/c/17950136739169608</t>
-  </si>
-  <si>
-    <t>https://www.instagram.com/p/DY2y0nlyyo1/c/17928198687318581</t>
-  </si>
-  <si>
-    <t>https://www.instagram.com/p/DY2y0nlyyo1/c/17952601112982084</t>
-  </si>
-  <si>
-    <t>https://www.instagram.com/p/DY2y0nlyyo1/c/18091811072608919</t>
-  </si>
-  <si>
-    <t>https://www.instagram.com/p/DY5JQwiEeiq/c/18091344725254984</t>
-  </si>
-  <si>
-    <t>https://www.instagram.com/p/DY5JQwiEeiq/c/17861475312635797</t>
-  </si>
-  <si>
-    <t>https://www.instagram.com/p/DY5JQwiEeiq/c/17992421969794446</t>
-  </si>
-  <si>
-    <t>https://www.instagram.com/p/DY5JQwiEeiq/c/18065414387686760</t>
-  </si>
-  <si>
-    <t>https://www.instagram.com/p/DY5JQwiEeiq/c/17975247609018419</t>
-  </si>
-  <si>
-    <t>17930061063295835</t>
-  </si>
-  <si>
-    <t>17950136739169608</t>
-  </si>
-  <si>
-    <t>17928198687318581</t>
-  </si>
-  <si>
-    <t>17952601112982084</t>
-  </si>
-  <si>
-    <t>18091811072608919</t>
-  </si>
-  <si>
-    <t>18091344725254984</t>
-  </si>
-  <si>
-    <t>17861475312635797</t>
-  </si>
-  <si>
-    <t>17992421969794446</t>
-  </si>
-  <si>
-    <t>18065414387686760</t>
-  </si>
-  <si>
-    <t>17975247609018419</t>
-  </si>
-  <si>
-    <t>esperava mais puc</t>
-  </si>
-  <si>
-    <t>Mentira que lançaram que é fake News KAKAKAKAKAK</t>
-  </si>
-  <si>
-    <t>A instituição q passa pano até pra assaltante</t>
-  </si>
-  <si>
-    <t>Então vcs estão tirando todas as vítimas pra doidos?</t>
-  </si>
-  <si>
-    <t>vocês devem estar de brincadeira, né?</t>
-  </si>
-  <si>
-    <t>sim obrigado PMMG.  Sem voces nada disso seria capaz. 🐽🐽🐷</t>
-  </si>
-  <si>
-    <t>Mas vai instalar catraca ou vai """"""instalar catraca"""""?</t>
-  </si>
-  <si>
-    <t>Deve ter umas duas décadas que q situação é a mesma!</t>
-  </si>
-  <si>
-    <t>vamos aguardar , + segurança será importante para todos !</t>
-  </si>
-  <si>
-    <t>até que enfim!!</t>
-  </si>
-  <si>
-    <t>cleo.sq</t>
-  </si>
-  <si>
-    <t>ingridsousamaquiadora</t>
-  </si>
-  <si>
-    <t>oanajulia_aaa</t>
-  </si>
-  <si>
-    <t>ggiovannac</t>
-  </si>
-  <si>
-    <t>joaoprivado_</t>
-  </si>
-  <si>
-    <t>lemarquescv</t>
-  </si>
-  <si>
-    <t>rodrigo.romero13</t>
-  </si>
-  <si>
-    <t>vital_kiko</t>
-  </si>
-  <si>
-    <t>gontijulia</t>
-  </si>
-  <si>
-    <t>https://scontent-ord5-2.cdninstagram.com/v/t51.82787-19/564421347_18107271349581839_3846479324225872497_n.jpg?stp=dst-jpg_s150x150_tt6&amp;_nc_cat=104&amp;ccb=7-5&amp;_nc_sid=f7ccc5&amp;efg=eyJ2ZW5jb2RlX3RhZyI6InByb2ZpbGVfcGljLnd3dy44MjguQzMifQ%3D%3D&amp;_nc_ohc=wdmI_ZD7AzEQ7kNvwFfln3a&amp;_nc_oc=AdpV5YEjcgpp6urIOJM4KRqJj0QXcX8kVHOwWpVATCOZbzkonjkIX5eDjUb1CBfxXZE&amp;_nc_zt=24&amp;_nc_ht=scontent-ord5-2.cdninstagram.com&amp;_nc_gid=NFKmeuilRk5_NljrInR2AQ&amp;_nc_ss=72a8c&amp;oh=00_Af6MX5qHDHOQPVdQyv156ET-h_1l-f5veR3_Elja8FnKBA&amp;oe=6A1E856A</t>
-  </si>
-  <si>
-    <t>https://scontent-ord5-2.cdninstagram.com/v/t51.82787-19/651897045_18419171566192007_5804309260263118662_n.jpg?stp=dst-jpg_s150x150_tt6&amp;_nc_cat=111&amp;ccb=7-5&amp;_nc_sid=f7ccc5&amp;efg=eyJ2ZW5jb2RlX3RhZyI6InByb2ZpbGVfcGljLnd3dy4xMDI0LkMzIn0%3D&amp;_nc_ohc=k-2HdImQjvUQ7kNvwEZGGW7&amp;_nc_oc=Adr2HyN3LMjueC1aFpN8NVPUbQv9Ym1-gc0na6uMNnmBcqM9exzpTMX8PI_Tv4n3rSc&amp;_nc_zt=24&amp;_nc_ht=scontent-ord5-2.cdninstagram.com&amp;_nc_gid=NFKmeuilRk5_NljrInR2AQ&amp;_nc_ss=72a8c&amp;oh=00_Af6phO2bkhaz4KENR1DYG835AXWvvJO0p8sJznEzoEDdAQ&amp;oe=6A1E7FB6</t>
-  </si>
-  <si>
-    <t>https://scontent-ord5-2.cdninstagram.com/v/t51.82787-19/514503002_17911250742157988_2317657929277158942_n.jpg?stp=dst-jpg_s150x150_tt6&amp;_nc_cat=103&amp;ccb=7-5&amp;_nc_sid=f7ccc5&amp;efg=eyJ2ZW5jb2RlX3RhZyI6InByb2ZpbGVfcGljLnd3dy4xMDgwLkMzIn0%3D&amp;_nc_ohc=2ONoLSAwn0YQ7kNvwF1Qkqs&amp;_nc_oc=AdoLBg74R3l9MDnj5EN_hojxYi841C9mDtVXW_pYcyEH8XqOMHIFNr7S5hOT5JZ5l3s&amp;_nc_zt=24&amp;_nc_ht=scontent-ord5-2.cdninstagram.com&amp;_nc_gid=NFKmeuilRk5_NljrInR2AQ&amp;_nc_ss=72a8c&amp;oh=00_Af4yHtH8sNMRqagwU--7QHU-rgIBZPktxk2SVH0WWyFsYA&amp;oe=6A1E87A3</t>
-  </si>
-  <si>
-    <t>https://scontent-ord5-2.cdninstagram.com/v/t51.2885-19/458976134_2057916541304864_4265730472601514728_n.jpg?stp=dst-jpg_s150x150_tt6&amp;_nc_cat=105&amp;ccb=7-5&amp;_nc_sid=f7ccc5&amp;efg=eyJ2ZW5jb2RlX3RhZyI6InByb2ZpbGVfcGljLnd3dy4xMDgwLkMzIn0%3D&amp;_nc_ohc=lMlfCRe5kzMQ7kNvwFM9XAr&amp;_nc_oc=AdqKQOu24WYPTTQLDSkk8t7qn07xJMIEASawiqRvhWPeAB3br8IoN6dC1e34q74YIBw&amp;_nc_zt=24&amp;_nc_ht=scontent-ord5-2.cdninstagram.com&amp;_nc_ss=72a8c&amp;oh=00_Af6n9hFwah6CJdI7IP7ZUblIDaZhx4VEp5grpYIYjQ1mrA&amp;oe=6A1E9C3F</t>
-  </si>
-  <si>
-    <t>https://scontent-lga3-1.cdninstagram.com/v/t51.2885-19/412710616_3447858782210471_273922732885924883_n.jpg?stp=dst-jpg_s150x150_tt6&amp;_nc_cat=110&amp;ccb=7-5&amp;_nc_sid=f7ccc5&amp;efg=eyJ2ZW5jb2RlX3RhZyI6InByb2ZpbGVfcGljLnd3dy4xMDgwLkMzIn0%3D&amp;_nc_ohc=1pvUrRm24a8Q7kNvwH3rFGR&amp;_nc_oc=AdoQqfDBK2kjB1aUs8k_SX9iIburSdC2WNghMyASytPbLcvKIVOkPtnHccuP-DzhSQA&amp;_nc_zt=24&amp;_nc_ht=scontent-lga3-1.cdninstagram.com&amp;_nc_ss=72a8c&amp;oh=00_Af7KAjq8awN9uiHxKo4NlppTEUJqtGxTRx8RkIWzVV9E9Q&amp;oe=6A1E9AEE</t>
-  </si>
-  <si>
-    <t>https://scontent-lga3-2.cdninstagram.com/v/t51.82787-19/654059159_18381633136091754_5012919991671065327_n.jpg?stp=dst-jpg_s150x150_tt6&amp;_nc_cat=100&amp;ccb=7-5&amp;_nc_sid=f7ccc5&amp;efg=eyJ2ZW5jb2RlX3RhZyI6InByb2ZpbGVfcGljLnd3dy4xMDgwLkMzIn0%3D&amp;_nc_ohc=5Fww9HfCgooQ7kNvwFh7DNV&amp;_nc_oc=AdoXMeOyURBiOnZGqk4yZj5QGZzMEQWAdDD9GnFcQSi2agmRs_Ottjr18Glo_QC3mpU&amp;_nc_zt=24&amp;_nc_ht=scontent-lga3-2.cdninstagram.com&amp;_nc_gid=mFFtzsJezkbFksziU-jr-w&amp;_nc_ss=72a8c&amp;oh=00_Af4US6djNezIbOByndrr29S1ihJDGpE1SnyaH35_V5NV6Q&amp;oe=6A1E75A8</t>
-  </si>
-  <si>
-    <t>https://scontent-lga3-2.cdninstagram.com/v/t51.82787-19/691911417_18581886802029369_3925767358805835986_n.jpg?stp=dst-jpg_s150x150_tt6&amp;_nc_cat=101&amp;ccb=7-5&amp;_nc_sid=f7ccc5&amp;efg=eyJ2ZW5jb2RlX3RhZyI6InByb2ZpbGVfcGljLnd3dy4xMDgwLkMzIn0%3D&amp;_nc_ohc=ESLj2OxoyHsQ7kNvwFkdxqZ&amp;_nc_oc=AdqT0UwHzXRCxNrM9aJ6bizMQI5OdAsl13K0cKy81iq9tBhSCylK_Yv3Wnw5zN_N3I4&amp;_nc_zt=24&amp;_nc_ht=scontent-lga3-2.cdninstagram.com&amp;_nc_gid=mFFtzsJezkbFksziU-jr-w&amp;_nc_ss=72a8c&amp;oh=00_Af5kHcHV9G128A0IN-Pq8ITs207Km4TXHina_wgaRGAdNQ&amp;oe=6A1EA797</t>
-  </si>
-  <si>
-    <t>https://scontent-lga3-2.cdninstagram.com/v/t51.2885-19/486758925_966180679028689_8159419035899772106_n.jpg?stp=dst-jpg_s150x150_tt6&amp;_nc_cat=100&amp;ccb=7-5&amp;_nc_sid=f7ccc5&amp;efg=eyJ2ZW5jb2RlX3RhZyI6InByb2ZpbGVfcGljLnd3dy4xMDgwLkMzIn0%3D&amp;_nc_ohc=Z-2U3YPPqOcQ7kNvwEZouI0&amp;_nc_oc=AdqcohAk8mlDXaN9VzgI53lTwcugx600cWrvQfDF4byrqwbRL6pc8UKnLBZzplGuUCE&amp;_nc_zt=24&amp;_nc_ht=scontent-lga3-2.cdninstagram.com&amp;_nc_ss=72a8c&amp;oh=00_Af5V5x8MaGlfUJ2Hf7Ug357aTQrmSHtBk4pwiPko4KyELA&amp;oe=6A1E7460</t>
-  </si>
-  <si>
-    <t>https://scontent-lga3-2.cdninstagram.com/v/t51.82787-19/648150350_18350975260228735_4039382149506883327_n.jpg?stp=dst-jpg_s150x150_tt6&amp;_nc_cat=101&amp;ccb=7-5&amp;_nc_sid=f7ccc5&amp;efg=eyJ2ZW5jb2RlX3RhZyI6InByb2ZpbGVfcGljLnd3dy4xMDgwLkMzIn0%3D&amp;_nc_ohc=oJsEPQZOJHEQ7kNvwGW1aun&amp;_nc_oc=AdqNTgiMCMo0DgdlHth_Gfp53nPT5ChfXBXRO0N-lE2wtzIUdgLE2wmnU6oFe47vtms&amp;_nc_zt=24&amp;_nc_ht=scontent-lga3-2.cdninstagram.com&amp;_nc_gid=mFFtzsJezkbFksziU-jr-w&amp;_nc_ss=72a8c&amp;oh=00_Af4onE3Ka9ZDC9UJVLyoC40T2TCEZ8irm0pSJ7TRcJCPMA&amp;oe=6A1E7B2E</t>
-  </si>
-  <si>
-    <t>2026-05-28T21:39:29.000Z</t>
-  </si>
-  <si>
-    <t>2026-05-28T21:12:03.000Z</t>
-  </si>
-  <si>
-    <t>2026-05-28T20:45:18.000Z</t>
-  </si>
-  <si>
-    <t>2026-05-28T20:44:52.000Z</t>
-  </si>
-  <si>
-    <t>2026-05-28T20:40:19.000Z</t>
-  </si>
-  <si>
-    <t>2026-05-28T21:36:09.000Z</t>
-  </si>
-  <si>
-    <t>2026-05-28T21:24:00.000Z</t>
-  </si>
-  <si>
-    <t>2026-05-28T21:12:15.000Z</t>
-  </si>
-  <si>
-    <t>2026-05-28T21:12:12.000Z</t>
-  </si>
-  <si>
-    <t>2026-05-28T21:09:45.000Z</t>
-  </si>
-  <si>
-    <t>{'username': 'cleo.sq', 'profile_pic_url': 'https://scontent-ord5-2.cdninstagram.com/v/t51.82787-19/564421347_18107271349581839_3846479324225872497_n.jpg?stp=dst-jpg_s150x150_tt6&amp;_nc_cat=104&amp;ccb=7-5&amp;_nc_sid=f7ccc5&amp;efg=eyJ2ZW5jb2RlX3RhZyI6InByb2ZpbGVfcGljLnd3dy44MjguQzMifQ%3D%3D&amp;_nc_ohc=wdmI_ZD7AzEQ7kNvwFfln3a&amp;_nc_oc=AdpV5YEjcgpp6urIOJM4KRqJj0QXcX8kVHOwWpVATCOZbzkonjkIX5eDjUb1CBfxXZE&amp;_nc_zt=24&amp;_nc_ht=scontent-ord5-2.cdninstagram.com&amp;_nc_gid=NFKmeuilRk5_NljrInR2AQ&amp;_nc_ss=72a8c&amp;oh=00_Af6MX5qHDHOQPVdQyv156ET-h_1l-f5veR3_Elja8FnKBA&amp;oe=6A1E856A', 'is_verified': False, 'id': '17395301838', 'fbid_v2': '17841417455154412', 'full_name': None, 'is_mentionable': None, 'is_private': None, 'profile_pic_id': None, 'latest_reel_media': None}</t>
-  </si>
-  <si>
-    <t>{'username': 'ingridsousamaquiadora', 'profile_pic_url': 'https://scontent-ord5-2.cdninstagram.com/v/t51.82787-19/651897045_18419171566192007_5804309260263118662_n.jpg?stp=dst-jpg_s150x150_tt6&amp;_nc_cat=111&amp;ccb=7-5&amp;_nc_sid=f7ccc5&amp;efg=eyJ2ZW5jb2RlX3RhZyI6InByb2ZpbGVfcGljLnd3dy4xMDI0LkMzIn0%3D&amp;_nc_ohc=k-2HdImQjvUQ7kNvwEZGGW7&amp;_nc_oc=Adr2HyN3LMjueC1aFpN8NVPUbQv9Ym1-gc0na6uMNnmBcqM9exzpTMX8PI_Tv4n3rSc&amp;_nc_zt=24&amp;_nc_ht=scontent-ord5-2.cdninstagram.com&amp;_nc_gid=NFKmeuilRk5_NljrInR2AQ&amp;_nc_ss=72a8c&amp;oh=00_Af6phO2bkhaz4KENR1DYG835AXWvvJO0p8sJznEzoEDdAQ&amp;oe=6A1E7FB6', 'is_verified': False, 'id': '5933872006', 'fbid_v2': '17841405760201734', 'full_name': None, 'is_mentionable': None, 'is_private': None, 'profile_pic_id': None, 'latest_reel_media': None}</t>
-  </si>
-  <si>
-    <t>{'username': 'oanajulia_aaa', 'profile_pic_url': 'https://scontent-ord5-2.cdninstagram.com/v/t51.82787-19/514503002_17911250742157988_2317657929277158942_n.jpg?stp=dst-jpg_s150x150_tt6&amp;_nc_cat=103&amp;ccb=7-5&amp;_nc_sid=f7ccc5&amp;efg=eyJ2ZW5jb2RlX3RhZyI6InByb2ZpbGVfcGljLnd3dy4xMDgwLkMzIn0%3D&amp;_nc_ohc=2ONoLSAwn0YQ7kNvwF1Qkqs&amp;_nc_oc=AdoLBg74R3l9MDnj5EN_hojxYi841C9mDtVXW_pYcyEH8XqOMHIFNr7S5hOT5JZ5l3s&amp;_nc_zt=24&amp;_nc_ht=scontent-ord5-2.cdninstagram.com&amp;_nc_gid=NFKmeuilRk5_NljrInR2AQ&amp;_nc_ss=72a8c&amp;oh=00_Af4yHtH8sNMRqagwU--7QHU-rgIBZPktxk2SVH0WWyFsYA&amp;oe=6A1E87A3', 'is_verified': False, 'id': '64582237987', 'fbid_v2': '17841464739612779', 'full_name': None, 'is_mentionable': None, 'is_private': None, 'profile_pic_id': None, 'latest_reel_media': None}</t>
-  </si>
-  <si>
-    <t>{'username': 'ggiovannac', 'profile_pic_url': 'https://scontent-ord5-2.cdninstagram.com/v/t51.2885-19/458976134_2057916541304864_4265730472601514728_n.jpg?stp=dst-jpg_s150x150_tt6&amp;_nc_cat=105&amp;ccb=7-5&amp;_nc_sid=f7ccc5&amp;efg=eyJ2ZW5jb2RlX3RhZyI6InByb2ZpbGVfcGljLnd3dy4xMDgwLkMzIn0%3D&amp;_nc_ohc=lMlfCRe5kzMQ7kNvwFM9XAr&amp;_nc_oc=AdqKQOu24WYPTTQLDSkk8t7qn07xJMIEASawiqRvhWPeAB3br8IoN6dC1e34q74YIBw&amp;_nc_zt=24&amp;_nc_ht=scontent-ord5-2.cdninstagram.com&amp;_nc_ss=72a8c&amp;oh=00_Af6n9hFwah6CJdI7IP7ZUblIDaZhx4VEp5grpYIYjQ1mrA&amp;oe=6A1E9C3F', 'is_verified': False, 'id': '990157599', 'fbid_v2': '17841400407985471', 'full_name': None, 'is_mentionable': None, 'is_private': None, 'profile_pic_id': None, 'latest_reel_media': None}</t>
-  </si>
-  <si>
-    <t>{'username': 'joaoprivado_', 'profile_pic_url': 'https://scontent-lga3-1.cdninstagram.com/v/t51.2885-19/412710616_3447858782210471_273922732885924883_n.jpg?stp=dst-jpg_s150x150_tt6&amp;_nc_cat=110&amp;ccb=7-5&amp;_nc_sid=f7ccc5&amp;efg=eyJ2ZW5jb2RlX3RhZyI6InByb2ZpbGVfcGljLnd3dy4xMDgwLkMzIn0%3D&amp;_nc_ohc=1pvUrRm24a8Q7kNvwH3rFGR&amp;_nc_oc=AdoQqfDBK2kjB1aUs8k_SX9iIburSdC2WNghMyASytPbLcvKIVOkPtnHccuP-DzhSQA&amp;_nc_zt=24&amp;_nc_ht=scontent-lga3-1.cdninstagram.com&amp;_nc_ss=72a8c&amp;oh=00_Af7KAjq8awN9uiHxKo4NlppTEUJqtGxTRx8RkIWzVV9E9Q&amp;oe=6A1E9AEE', 'is_verified': False, 'id': '6807727160', 'fbid_v2': '17841406934810965', 'full_name': None, 'is_mentionable': None, 'is_private': None, 'profile_pic_id': None, 'latest_reel_media': None}</t>
-  </si>
-  <si>
-    <t>{'username': 'lemarquescv', 'profile_pic_url': 'https://scontent-lga3-2.cdninstagram.com/v/t51.82787-19/654059159_18381633136091754_5012919991671065327_n.jpg?stp=dst-jpg_s150x150_tt6&amp;_nc_cat=100&amp;ccb=7-5&amp;_nc_sid=f7ccc5&amp;efg=eyJ2ZW5jb2RlX3RhZyI6InByb2ZpbGVfcGljLnd3dy4xMDgwLkMzIn0%3D&amp;_nc_ohc=5Fww9HfCgooQ7kNvwFh7DNV&amp;_nc_oc=AdoXMeOyURBiOnZGqk4yZj5QGZzMEQWAdDD9GnFcQSi2agmRs_Ottjr18Glo_QC3mpU&amp;_nc_zt=24&amp;_nc_ht=scontent-lga3-2.cdninstagram.com&amp;_nc_gid=mFFtzsJezkbFksziU-jr-w&amp;_nc_ss=72a8c&amp;oh=00_Af4US6djNezIbOByndrr29S1ihJDGpE1SnyaH35_V5NV6Q&amp;oe=6A1E75A8', 'is_verified': False, 'id': '2714443753', 'fbid_v2': '17841402752599305', 'full_name': None, 'is_mentionable': None, 'is_private': None, 'profile_pic_id': None, 'latest_reel_media': None}</t>
-  </si>
-  <si>
-    <t>{'username': 'rodrigo.romero13', 'profile_pic_url': 'https://scontent-lga3-2.cdninstagram.com/v/t51.82787-19/691911417_18581886802029369_3925767358805835986_n.jpg?stp=dst-jpg_s150x150_tt6&amp;_nc_cat=101&amp;ccb=7-5&amp;_nc_sid=f7ccc5&amp;efg=eyJ2ZW5jb2RlX3RhZyI6InByb2ZpbGVfcGljLnd3dy4xMDgwLkMzIn0%3D&amp;_nc_ohc=ESLj2OxoyHsQ7kNvwFkdxqZ&amp;_nc_oc=AdqT0UwHzXRCxNrM9aJ6bizMQI5OdAsl13K0cKy81iq9tBhSCylK_Yv3Wnw5zN_N3I4&amp;_nc_zt=24&amp;_nc_ht=scontent-lga3-2.cdninstagram.com&amp;_nc_gid=mFFtzsJezkbFksziU-jr-w&amp;_nc_ss=72a8c&amp;oh=00_Af5kHcHV9G128A0IN-Pq8ITs207Km4TXHina_wgaRGAdNQ&amp;oe=6A1EA797', 'is_verified': False, 'id': '1137949368', 'fbid_v2': '17841400881057780', 'full_name': None, 'is_mentionable': None, 'is_private': None, 'profile_pic_id': None, 'latest_reel_media': None}</t>
-  </si>
-  <si>
-    <t>{'username': 'vital_kiko', 'profile_pic_url': 'https://scontent-lga3-2.cdninstagram.com/v/t51.2885-19/486758925_966180679028689_8159419035899772106_n.jpg?stp=dst-jpg_s150x150_tt6&amp;_nc_cat=100&amp;ccb=7-5&amp;_nc_sid=f7ccc5&amp;efg=eyJ2ZW5jb2RlX3RhZyI6InByb2ZpbGVfcGljLnd3dy4xMDgwLkMzIn0%3D&amp;_nc_ohc=Z-2U3YPPqOcQ7kNvwEZouI0&amp;_nc_oc=AdqcohAk8mlDXaN9VzgI53lTwcugx600cWrvQfDF4byrqwbRL6pc8UKnLBZzplGuUCE&amp;_nc_zt=24&amp;_nc_ht=scontent-lga3-2.cdninstagram.com&amp;_nc_ss=72a8c&amp;oh=00_Af5V5x8MaGlfUJ2Hf7Ug357aTQrmSHtBk4pwiPko4KyELA&amp;oe=6A1E7460', 'is_verified': False, 'id': '44181163545', 'fbid_v2': '17841444266352645', 'full_name': None, 'is_mentionable': None, 'is_private': None, 'profile_pic_id': None, 'latest_reel_media': None}</t>
-  </si>
-  <si>
-    <t>{'username': 'gontijulia', 'profile_pic_url': 'https://scontent-lga3-2.cdninstagram.com/v/t51.82787-19/648150350_18350975260228735_4039382149506883327_n.jpg?stp=dst-jpg_s150x150_tt6&amp;_nc_cat=101&amp;ccb=7-5&amp;_nc_sid=f7ccc5&amp;efg=eyJ2ZW5jb2RlX3RhZyI6InByb2ZpbGVfcGljLnd3dy4xMDgwLkMzIn0%3D&amp;_nc_ohc=oJsEPQZOJHEQ7kNvwGW1aun&amp;_nc_oc=AdqNTgiMCMo0DgdlHth_Gfp53nPT5ChfXBXRO0N-lE2wtzIUdgLE2wmnU6oFe47vtms&amp;_nc_zt=24&amp;_nc_ht=scontent-lga3-2.cdninstagram.com&amp;_nc_gid=mFFtzsJezkbFksziU-jr-w&amp;_nc_ss=72a8c&amp;oh=00_Af4onE3Ka9ZDC9UJVLyoC40T2TCEZ8irm0pSJ7TRcJCPMA&amp;oe=6A1E7B2E', 'is_verified': False, 'id': '6804596734', 'fbid_v2': '17841406862030574', 'full_name': None, 'is_mentionable': None, 'is_private': None, 'profile_pic_id': None, 'latest_reel_media': None}</t>
+    <t>https://www.instagram.com/p/DY5JQwiEeiq/c/18106633885940623</t>
+  </si>
+  <si>
+    <t>https://www.instagram.com/p/DY5JQwiEeiq/c/18078296204222063</t>
+  </si>
+  <si>
+    <t>https://www.instagram.com/p/DY5JQwiEeiq/c/18089660867630448</t>
+  </si>
+  <si>
+    <t>https://www.instagram.com/p/DY5JQwiEeiq/c/18157379752456658</t>
+  </si>
+  <si>
+    <t>https://www.instagram.com/p/DY5JQwiEeiq/c/17989044197995436</t>
+  </si>
+  <si>
+    <t>https://www.instagram.com/p/DY2y0nlyyo1/c/18547118032070028</t>
+  </si>
+  <si>
+    <t>https://www.instagram.com/p/DY2y0nlyyo1/c/18115328398634083</t>
+  </si>
+  <si>
+    <t>https://www.instagram.com/p/DY2y0nlyyo1/c/17878318605605833</t>
+  </si>
+  <si>
+    <t>https://www.instagram.com/p/DY2y0nlyyo1/c/18395105302083069</t>
+  </si>
+  <si>
+    <t>https://www.instagram.com/p/DY2y0nlyyo1/c/17967954975112796</t>
+  </si>
+  <si>
+    <t>18106633885940623</t>
+  </si>
+  <si>
+    <t>18078296204222063</t>
+  </si>
+  <si>
+    <t>18089660867630448</t>
+  </si>
+  <si>
+    <t>18157379752456658</t>
+  </si>
+  <si>
+    <t>17989044197995436</t>
+  </si>
+  <si>
+    <t>18547118032070028</t>
+  </si>
+  <si>
+    <t>18115328398634083</t>
+  </si>
+  <si>
+    <t>17878318605605833</t>
+  </si>
+  <si>
+    <t>18395105302083069</t>
+  </si>
+  <si>
+    <t>17967954975112796</t>
+  </si>
+  <si>
+    <t>Ué o último pronunciamento dizia que nao havia aumento nos crimes... agora estao sendo tomadas medidas??</t>
+  </si>
+  <si>
+    <t>Não temos segurança nem na universidade. PARTICULAR!!! ABSURDO DEVE TA BARATO AS MENSALIDADES!</t>
+  </si>
+  <si>
+    <t>Hoje mais dois alunos foram assaltados em frente o coreu burguer. Pagamos 2k de mensalidade pra isso?</t>
+  </si>
+  <si>
+    <t>Catraca ou sabor catraca?</t>
+  </si>
+  <si>
+    <t>Que bom que foram começadas  algumas propostas de mudanças,esperamos que os resultados sejam mais próximos possíveis, não só os alunos mas funcionários também passavam por essa situação,como mãe fico um pouco mais aliviada.obrigada pelas iniciativas.</t>
+  </si>
+  <si>
+    <t>Façam o L imediatamente</t>
+  </si>
+  <si>
+    <t>estamos vivendo em um mundo paralelo, não acredito que li isso!</t>
+  </si>
+  <si>
+    <t>Vocês gastam horrores pra fazer obras e pinturas desnecessárias e fechar partes da faculdade por um bom tempo, mas não podem investir tempo e dinheiro em segurança do campus? Entra quem quiser naquele lugar, não tem como fingir que se importam com segurança e falta de verba não é, é falta de vontade.</t>
+  </si>
+  <si>
+    <t>Estão dizendo que as vítimas estão mentindo? O que ganharia mulheres universitárias em mentir sobre uma onda de assaltos? Não foram uma, ou duas estudantes isoladas... há videos dos ocorridos próximo ao campus, há também relatos. Descredibilizar não nos leva à lugar algum.</t>
+  </si>
+  <si>
+    <t>Vergonhoso em uma universidade particular do nível da PUC Minas não ser exigido verificação de pessoas e monitorização, nem que seja por meio de catraca como no complexo esportivo!</t>
+  </si>
+  <si>
+    <t>luciofnaves</t>
+  </si>
+  <si>
+    <t>arthrvg</t>
+  </si>
+  <si>
+    <t>barbaralgon</t>
+  </si>
+  <si>
+    <t>ivy_tavares7</t>
+  </si>
+  <si>
+    <t>naybc89</t>
+  </si>
+  <si>
+    <t>millenascc</t>
+  </si>
+  <si>
+    <t>deboracsigaud</t>
+  </si>
+  <si>
+    <t>alic_quirino</t>
+  </si>
+  <si>
+    <t>anagiulialiberato</t>
+  </si>
+  <si>
+    <t>https://scontent-dfw5-1.cdninstagram.com/v/t51.82787-19/532180906_18520829407004424_4875931443338706572_n.jpg?stp=dst-jpg_s150x150_tt6&amp;_nc_cat=111&amp;ccb=7-5&amp;_nc_sid=f7ccc5&amp;efg=eyJ2ZW5jb2RlX3RhZyI6InByb2ZpbGVfcGljLnd3dy45NTguQzMifQ%3D%3D&amp;_nc_ohc=QBm1wA3UzeQQ7kNvwEUAMnD&amp;_nc_oc=AdpEbjTyfWyg3iyy1S2_wADzTXYHWKIcBlpX54lXkAZeAHRZaQp6SPE2XBgs--H40OA&amp;_nc_zt=24&amp;_nc_ht=scontent-dfw5-1.cdninstagram.com&amp;_nc_gid=6bndXB_NYJWtedf4oCeSZg&amp;_nc_ss=72a8c&amp;oh=00_Af6Wx2gxrNabiFP8z6eWo7oyuSVpO3rNcQlhpVBJZS-aPg&amp;oe=6A1EE9AE</t>
+  </si>
+  <si>
+    <t>https://scontent-dfw6-1.cdninstagram.com/v/t51.82787-19/522643831_18522048226038057_789159453189720233_n.jpg?stp=dst-jpg_s150x150_tt6&amp;_nc_cat=103&amp;ccb=7-5&amp;_nc_sid=f7ccc5&amp;efg=eyJ2ZW5jb2RlX3RhZyI6InByb2ZpbGVfcGljLnd3dy4xMDgwLkMzIn0%3D&amp;_nc_ohc=hyOX21yJGE4Q7kNvwFt41y1&amp;_nc_oc=AdoZk5HcqyC4yd_yrfzppXHEfvaXLjkZ9ujJTv47WjNQbDzB7SjmKu6MbXTqprek-d4&amp;_nc_zt=24&amp;_nc_ht=scontent-dfw6-1.cdninstagram.com&amp;_nc_gid=6bndXB_NYJWtedf4oCeSZg&amp;_nc_ss=72a8c&amp;oh=00_Af4wQ2r1n3e2ExlNl9L0gePOv1lkMji73cbrGQeYMfjB_w&amp;oe=6A1EC653</t>
+  </si>
+  <si>
+    <t>https://scontent-dfw5-2.cdninstagram.com/v/t51.82787-19/705981688_18594144139037165_1618853508786384328_n.jpg?stp=dst-jpg_s150x150_tt6&amp;_nc_cat=100&amp;ccb=7-5&amp;_nc_sid=f7ccc5&amp;efg=eyJ2ZW5jb2RlX3RhZyI6InByb2ZpbGVfcGljLnd3dy44ODMuQzMifQ%3D%3D&amp;_nc_ohc=41ALjYZVKdUQ7kNvwGIx8hR&amp;_nc_oc=Adr1gbl5DUfvbw3H8CgUWsaN_gzxG-HPm0lODksVJaEtMF3TbY-GzKW1ScTTyCO5HQA&amp;_nc_zt=24&amp;_nc_ht=scontent-dfw5-2.cdninstagram.com&amp;_nc_gid=6bndXB_NYJWtedf4oCeSZg&amp;_nc_ss=72a8c&amp;oh=00_Af4B4kWNISCRAWO1krXAlOG5qGNRR6Qjtexx2Q4zNcF0lw&amp;oe=6A1EB425</t>
+  </si>
+  <si>
+    <t>https://scontent-dfw5-1.cdninstagram.com/v/t51.75761-19/499676212_18505554592030169_5411618968558129339_n.jpg?stp=dst-jpg_s150x150_tt6&amp;_nc_cat=111&amp;ccb=7-5&amp;_nc_sid=f7ccc5&amp;efg=eyJ2ZW5jb2RlX3RhZyI6InByb2ZpbGVfcGljLnd3dy4xMDgwLkMzIn0%3D&amp;_nc_ohc=RPaUAp0KL3kQ7kNvwG13Hw6&amp;_nc_oc=Adqlz2NwGjyIhBVQwTZw1bYwHXRbtZpf-Zyo7uoO26bNHzqec7kJcbD2_PhOLtL_lLo&amp;_nc_zt=24&amp;_nc_ht=scontent-dfw5-1.cdninstagram.com&amp;_nc_gid=6bndXB_NYJWtedf4oCeSZg&amp;_nc_ss=72a8c&amp;oh=00_Af7hQ-avKrh1ZovfgjX04odZ91fCybFfDrQKRVIpaKNZTA&amp;oe=6A1EB1FE</t>
+  </si>
+  <si>
+    <t>https://scontent-lax3-1.cdninstagram.com/v/t51.82787-19/617607685_18552756436023707_1422186455618419422_n.jpg?stp=dst-jpg_s150x150_tt6&amp;_nc_cat=104&amp;ccb=7-5&amp;_nc_sid=f7ccc5&amp;efg=eyJ2ZW5jb2RlX3RhZyI6InByb2ZpbGVfcGljLnd3dy40MzEuQzMifQ%3D%3D&amp;_nc_ohc=wijU7KyiX4YQ7kNvwF4uRgs&amp;_nc_oc=AdqYJejxOI6nugEAjC_pnwEqJb6CE5mGZ6-stmmgsoCGY9a-QZh1ep_QAvPzyra8OMQ&amp;_nc_zt=24&amp;_nc_ht=scontent-lax3-1.cdninstagram.com&amp;_nc_gid=AB75SZJbTl-V2pBFLFZaTQ&amp;_nc_ss=72689&amp;oh=00_Af6RvAPniH-LwWM3x3wRX4cjubWNWJQbA5-UO7OmIRJURQ&amp;oe=6A1ED466</t>
+  </si>
+  <si>
+    <t>https://scontent-lax3-1.cdninstagram.com/v/t51.75761-19/494943345_18171624601335760_823979804544109417_n.jpg?stp=dst-jpg_s150x150_tt6&amp;_nc_cat=108&amp;ccb=7-5&amp;_nc_sid=f7ccc5&amp;efg=eyJ2ZW5jb2RlX3RhZyI6InByb2ZpbGVfcGljLnd3dy4xMDgwLkMzIn0%3D&amp;_nc_ohc=reqcgJcGq0cQ7kNvwGakWhh&amp;_nc_oc=AdqDmp315D84K-Kbz4yKPsBdoK-s0xdKFtOEWAa10Qy-A-fwBMyV5mQoqxw22rSJZHE&amp;_nc_zt=24&amp;_nc_ht=scontent-lax3-1.cdninstagram.com&amp;_nc_gid=AB75SZJbTl-V2pBFLFZaTQ&amp;_nc_ss=72689&amp;oh=00_Af7xIIdy8DU4OSHWwERQKRSkT8LCyea19DB7SCDiqid2gw&amp;oe=6A1EB491</t>
+  </si>
+  <si>
+    <t>https://scontent-lax3-1.cdninstagram.com/v/t51.82787-19/649210535_18448352116128501_2624709667249038068_n.jpg?stp=dst-jpg_s150x150_tt6&amp;_nc_cat=109&amp;ccb=7-5&amp;_nc_sid=f7ccc5&amp;efg=eyJ2ZW5jb2RlX3RhZyI6InByb2ZpbGVfcGljLnd3dy4xMDgwLkMzIn0%3D&amp;_nc_ohc=ESm2mcqHxa8Q7kNvwEDqw99&amp;_nc_oc=Adp6TnMEKFa2oW53NG1YsxoaGm05LZsdlj84Cq7-ewHtLX9zFY3IpNTQneAEdd5D350&amp;_nc_zt=24&amp;_nc_ht=scontent-lax3-1.cdninstagram.com&amp;_nc_gid=AB75SZJbTl-V2pBFLFZaTQ&amp;_nc_ss=72689&amp;oh=00_Af7nWz8RrvG5msc4tneaGTAUZWj1CwAnqIMIRCtzY02tAw&amp;oe=6A1ED882</t>
+  </si>
+  <si>
+    <t>https://scontent-lax3-1.cdninstagram.com/v/t51.82787-19/706583236_18421012582132902_883757664613422855_n.jpg?stp=dst-jpg_s150x150_tt6&amp;_nc_cat=109&amp;ccb=7-5&amp;_nc_sid=f7ccc5&amp;efg=eyJ2ZW5jb2RlX3RhZyI6InByb2ZpbGVfcGljLnd3dy4xMDgwLkMzIn0%3D&amp;_nc_ohc=DBfQYqDwKJoQ7kNvwGSpp3A&amp;_nc_oc=AdrTRi4fB31A3TC0ebz__OPT2olB_rYiNsTiSnhWKW0ylLI8mQljMGdcvDWLxZu28xI&amp;_nc_zt=24&amp;_nc_ht=scontent-lax3-1.cdninstagram.com&amp;_nc_gid=AB75SZJbTl-V2pBFLFZaTQ&amp;_nc_ss=72689&amp;oh=00_Af6oRHA6-ZpGXOgczcE5CLZZAglkVKPgx4msfBSYG_mZcw&amp;oe=6A1ED205</t>
+  </si>
+  <si>
+    <t>https://scontent-lax3-1.cdninstagram.com/v/t51.82787-19/615681840_18007275203829818_8813883761389566737_n.jpg?stp=dst-jpg_s150x150_tt6&amp;_nc_cat=108&amp;ccb=7-5&amp;_nc_sid=f7ccc5&amp;efg=eyJ2ZW5jb2RlX3RhZyI6InByb2ZpbGVfcGljLnd3dy4xMDgwLkMzIn0%3D&amp;_nc_ohc=RkqtY10-2qQQ7kNvwFBJmv5&amp;_nc_oc=Adpt9e90EUZm8jeK7hoPCq9fMODNpOZIVD3tDSVD7OUw2KfXX3SWiumCvgujPyg8qp0&amp;_nc_zt=24&amp;_nc_ht=scontent-lax3-1.cdninstagram.com&amp;_nc_gid=AB75SZJbTl-V2pBFLFZaTQ&amp;_nc_ss=72689&amp;oh=00_Af4gUXlvtPn4wJmf03PoNJWpzornkEft6Up-sZaTkm23Gw&amp;oe=6A1EB64B</t>
+  </si>
+  <si>
+    <t>2026-05-29T02:17:42.000Z</t>
+  </si>
+  <si>
+    <t>2026-05-29T02:14:11.000Z</t>
+  </si>
+  <si>
+    <t>2026-05-29T02:13:47.000Z</t>
+  </si>
+  <si>
+    <t>2026-05-29T02:13:07.000Z</t>
+  </si>
+  <si>
+    <t>2026-05-29T01:15:08.000Z</t>
+  </si>
+  <si>
+    <t>2026-05-29T01:47:42.000Z</t>
+  </si>
+  <si>
+    <t>2026-05-29T01:16:38.000Z</t>
+  </si>
+  <si>
+    <t>2026-05-29T00:57:41.000Z</t>
+  </si>
+  <si>
+    <t>2026-05-29T00:10:03.000Z</t>
+  </si>
+  <si>
+    <t>2026-05-28T22:54:47.000Z</t>
+  </si>
+  <si>
+    <t>{'username': 'luciofnaves', 'profile_pic_url': 'https://scontent-dfw5-1.cdninstagram.com/v/t51.82787-19/532180906_18520829407004424_4875931443338706572_n.jpg?stp=dst-jpg_s150x150_tt6&amp;_nc_cat=111&amp;ccb=7-5&amp;_nc_sid=f7ccc5&amp;efg=eyJ2ZW5jb2RlX3RhZyI6InByb2ZpbGVfcGljLnd3dy45NTguQzMifQ%3D%3D&amp;_nc_ohc=QBm1wA3UzeQQ7kNvwEUAMnD&amp;_nc_oc=AdpEbjTyfWyg3iyy1S2_wADzTXYHWKIcBlpX54lXkAZeAHRZaQp6SPE2XBgs--H40OA&amp;_nc_zt=24&amp;_nc_ht=scontent-dfw5-1.cdninstagram.com&amp;_nc_gid=6bndXB_NYJWtedf4oCeSZg&amp;_nc_ss=72a8c&amp;oh=00_Af6Wx2gxrNabiFP8z6eWo7oyuSVpO3rNcQlhpVBJZS-aPg&amp;oe=6A1EE9AE', 'is_verified': False, 'id': '237764423', 'fbid_v2': '17841400132693715', 'full_name': None, 'is_mentionable': None, 'is_private': None, 'profile_pic_id': None, 'latest_reel_media': None}</t>
+  </si>
+  <si>
+    <t>{'username': 'arthrvg', 'profile_pic_url': 'https://scontent-dfw6-1.cdninstagram.com/v/t51.82787-19/522643831_18522048226038057_789159453189720233_n.jpg?stp=dst-jpg_s150x150_tt6&amp;_nc_cat=103&amp;ccb=7-5&amp;_nc_sid=f7ccc5&amp;efg=eyJ2ZW5jb2RlX3RhZyI6InByb2ZpbGVfcGljLnd3dy4xMDgwLkMzIn0%3D&amp;_nc_ohc=hyOX21yJGE4Q7kNvwFt41y1&amp;_nc_oc=AdoZk5HcqyC4yd_yrfzppXHEfvaXLjkZ9ujJTv47WjNQbDzB7SjmKu6MbXTqprek-d4&amp;_nc_zt=24&amp;_nc_ht=scontent-dfw6-1.cdninstagram.com&amp;_nc_gid=6bndXB_NYJWtedf4oCeSZg&amp;_nc_ss=72a8c&amp;oh=00_Af4wQ2r1n3e2ExlNl9L0gePOv1lkMji73cbrGQeYMfjB_w&amp;oe=6A1EC653', 'is_verified': False, 'id': '1692390056', 'fbid_v2': '17841401141706443', 'full_name': None, 'is_mentionable': None, 'is_private': None, 'profile_pic_id': None, 'latest_reel_media': None}</t>
+  </si>
+  <si>
+    <t>{'username': 'barbaralgon', 'profile_pic_url': 'https://scontent-dfw5-2.cdninstagram.com/v/t51.82787-19/705981688_18594144139037165_1618853508786384328_n.jpg?stp=dst-jpg_s150x150_tt6&amp;_nc_cat=100&amp;ccb=7-5&amp;_nc_sid=f7ccc5&amp;efg=eyJ2ZW5jb2RlX3RhZyI6InByb2ZpbGVfcGljLnd3dy44ODMuQzMifQ%3D%3D&amp;_nc_ohc=41ALjYZVKdUQ7kNvwGIx8hR&amp;_nc_oc=Adr1gbl5DUfvbw3H8CgUWsaN_gzxG-HPm0lODksVJaEtMF3TbY-GzKW1ScTTyCO5HQA&amp;_nc_zt=24&amp;_nc_ht=scontent-dfw5-2.cdninstagram.com&amp;_nc_gid=6bndXB_NYJWtedf4oCeSZg&amp;_nc_ss=72a8c&amp;oh=00_Af4B4kWNISCRAWO1krXAlOG5qGNRR6Qjtexx2Q4zNcF0lw&amp;oe=6A1EB425', 'is_verified': False, 'id': '286949164', 'fbid_v2': '17841401114924483', 'full_name': None, 'is_mentionable': None, 'is_private': None, 'profile_pic_id': None, 'latest_reel_media': None}</t>
+  </si>
+  <si>
+    <t>{'username': 'ivy_tavares7', 'profile_pic_url': 'https://scontent-dfw5-1.cdninstagram.com/v/t51.75761-19/499676212_18505554592030169_5411618968558129339_n.jpg?stp=dst-jpg_s150x150_tt6&amp;_nc_cat=111&amp;ccb=7-5&amp;_nc_sid=f7ccc5&amp;efg=eyJ2ZW5jb2RlX3RhZyI6InByb2ZpbGVfcGljLnd3dy4xMDgwLkMzIn0%3D&amp;_nc_ohc=RPaUAp0KL3kQ7kNvwG13Hw6&amp;_nc_oc=Adqlz2NwGjyIhBVQwTZw1bYwHXRbtZpf-Zyo7uoO26bNHzqec7kJcbD2_PhOLtL_lLo&amp;_nc_zt=24&amp;_nc_ht=scontent-dfw5-1.cdninstagram.com&amp;_nc_gid=6bndXB_NYJWtedf4oCeSZg&amp;_nc_ss=72a8c&amp;oh=00_Af7hQ-avKrh1ZovfgjX04odZ91fCybFfDrQKRVIpaKNZTA&amp;oe=6A1EB1FE', 'is_verified': False, 'id': '1324062168', 'fbid_v2': '17841400905060688', 'full_name': None, 'is_mentionable': None, 'is_private': None, 'profile_pic_id': None, 'latest_reel_media': None}</t>
+  </si>
+  <si>
+    <t>{'username': 'naybc89', 'profile_pic_url': 'https://scontent-lax3-1.cdninstagram.com/v/t51.82787-19/617607685_18552756436023707_1422186455618419422_n.jpg?stp=dst-jpg_s150x150_tt6&amp;_nc_cat=104&amp;ccb=7-5&amp;_nc_sid=f7ccc5&amp;efg=eyJ2ZW5jb2RlX3RhZyI6InByb2ZpbGVfcGljLnd3dy40MzEuQzMifQ%3D%3D&amp;_nc_ohc=wijU7KyiX4YQ7kNvwF4uRgs&amp;_nc_oc=AdqYJejxOI6nugEAjC_pnwEqJb6CE5mGZ6-stmmgsoCGY9a-QZh1ep_QAvPzyra8OMQ&amp;_nc_zt=24&amp;_nc_ht=scontent-lax3-1.cdninstagram.com&amp;_nc_gid=AB75SZJbTl-V2pBFLFZaTQ&amp;_nc_ss=72689&amp;oh=00_Af6RvAPniH-LwWM3x3wRX4cjubWNWJQbA5-UO7OmIRJURQ&amp;oe=6A1ED466', 'is_verified': False, 'id': '9751706', 'fbid_v2': '17841400711180152', 'full_name': None, 'is_mentionable': None, 'is_private': None, 'profile_pic_id': None, 'latest_reel_media': None}</t>
+  </si>
+  <si>
+    <t>{'username': 'millenascc', 'profile_pic_url': 'https://scontent-lax3-1.cdninstagram.com/v/t51.75761-19/494943345_18171624601335760_823979804544109417_n.jpg?stp=dst-jpg_s150x150_tt6&amp;_nc_cat=108&amp;ccb=7-5&amp;_nc_sid=f7ccc5&amp;efg=eyJ2ZW5jb2RlX3RhZyI6InByb2ZpbGVfcGljLnd3dy4xMDgwLkMzIn0%3D&amp;_nc_ohc=reqcgJcGq0cQ7kNvwGakWhh&amp;_nc_oc=AdqDmp315D84K-Kbz4yKPsBdoK-s0xdKFtOEWAa10Qy-A-fwBMyV5mQoqxw22rSJZHE&amp;_nc_zt=24&amp;_nc_ht=scontent-lax3-1.cdninstagram.com&amp;_nc_gid=AB75SZJbTl-V2pBFLFZaTQ&amp;_nc_ss=72689&amp;oh=00_Af7xIIdy8DU4OSHWwERQKRSkT8LCyea19DB7SCDiqid2gw&amp;oe=6A1EB491', 'is_verified': False, 'id': '9842511759', 'fbid_v2': '17841410072770313', 'full_name': None, 'is_mentionable': None, 'is_private': None, 'profile_pic_id': None, 'latest_reel_media': None}</t>
+  </si>
+  <si>
+    <t>{'username': 'deboracsigaud', 'profile_pic_url': 'https://scontent-lax3-1.cdninstagram.com/v/t51.82787-19/649210535_18448352116128501_2624709667249038068_n.jpg?stp=dst-jpg_s150x150_tt6&amp;_nc_cat=109&amp;ccb=7-5&amp;_nc_sid=f7ccc5&amp;efg=eyJ2ZW5jb2RlX3RhZyI6InByb2ZpbGVfcGljLnd3dy4xMDgwLkMzIn0%3D&amp;_nc_ohc=ESm2mcqHxa8Q7kNvwEDqw99&amp;_nc_oc=Adp6TnMEKFa2oW53NG1YsxoaGm05LZsdlj84Cq7-ewHtLX9zFY3IpNTQneAEdd5D350&amp;_nc_zt=24&amp;_nc_ht=scontent-lax3-1.cdninstagram.com&amp;_nc_gid=AB75SZJbTl-V2pBFLFZaTQ&amp;_nc_ss=72689&amp;oh=00_Af7nWz8RrvG5msc4tneaGTAUZWj1CwAnqIMIRCtzY02tAw&amp;oe=6A1ED882', 'is_verified': False, 'id': '4052392500', 'fbid_v2': '17841403855026549', 'full_name': None, 'is_mentionable': None, 'is_private': None, 'profile_pic_id': None, 'latest_reel_media': None}</t>
+  </si>
+  <si>
+    <t>{'username': 'alic_quirino', 'profile_pic_url': 'https://scontent-lax3-1.cdninstagram.com/v/t51.82787-19/706583236_18421012582132902_883757664613422855_n.jpg?stp=dst-jpg_s150x150_tt6&amp;_nc_cat=109&amp;ccb=7-5&amp;_nc_sid=f7ccc5&amp;efg=eyJ2ZW5jb2RlX3RhZyI6InByb2ZpbGVfcGljLnd3dy4xMDgwLkMzIn0%3D&amp;_nc_ohc=DBfQYqDwKJoQ7kNvwGSpp3A&amp;_nc_oc=AdrTRi4fB31A3TC0ebz__OPT2olB_rYiNsTiSnhWKW0ylLI8mQljMGdcvDWLxZu28xI&amp;_nc_zt=24&amp;_nc_ht=scontent-lax3-1.cdninstagram.com&amp;_nc_gid=AB75SZJbTl-V2pBFLFZaTQ&amp;_nc_ss=72689&amp;oh=00_Af6oRHA6-ZpGXOgczcE5CLZZAglkVKPgx4msfBSYG_mZcw&amp;oe=6A1ED205', 'is_verified': False, 'id': '4040756901', 'fbid_v2': '17841403987055094', 'full_name': None, 'is_mentionable': None, 'is_private': None, 'profile_pic_id': None, 'latest_reel_media': None}</t>
+  </si>
+  <si>
+    <t>{'username': 'anagiulialiberato', 'profile_pic_url': 'https://scontent-lax3-1.cdninstagram.com/v/t51.82787-19/615681840_18007275203829818_8813883761389566737_n.jpg?stp=dst-jpg_s150x150_tt6&amp;_nc_cat=108&amp;ccb=7-5&amp;_nc_sid=f7ccc5&amp;efg=eyJ2ZW5jb2RlX3RhZyI6InByb2ZpbGVfcGljLnd3dy4xMDgwLkMzIn0%3D&amp;_nc_ohc=RkqtY10-2qQQ7kNvwFBJmv5&amp;_nc_oc=Adpt9e90EUZm8jeK7hoPCq9fMODNpOZIVD3tDSVD7OUw2KfXX3SWiumCvgujPyg8qp0&amp;_nc_zt=24&amp;_nc_ht=scontent-lax3-1.cdninstagram.com&amp;_nc_gid=AB75SZJbTl-V2pBFLFZaTQ&amp;_nc_ss=72689&amp;oh=00_Af4gUXlvtPn4wJmf03PoNJWpzornkEft6Up-sZaTkm23Gw&amp;oe=6A1EB64B', 'is_verified': False, 'id': '54831765817', 'fbid_v2': '17841454894523970', 'full_name': None, 'is_mentionable': None, 'is_private': None, 'profile_pic_id': None, 'latest_reel_media': None}</t>
   </si>
 </sst>
 </file>
@@ -734,10 +734,10 @@
         <v>35</v>
       </c>
       <c r="E4" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="G4" t="s">
         <v>63</v>
@@ -746,7 +746,7 @@
         <v>0</v>
       </c>
       <c r="K4" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="5" spans="1:11">
@@ -859,7 +859,7 @@
         <v>67</v>
       </c>
       <c r="J8">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="K8" t="s">
         <v>76</v>

</xml_diff>